<commit_message>
Implementando mejoras en el diseño de producto, añadiendo scroll de cantidad a comprar
</commit_message>
<xml_diff>
--- a/DataCSV/Productos.xlsx
+++ b/DataCSV/Productos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JOSE\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PAGINA-WEB\PaginaVentas\DataCSV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C42D4F4-42B1-4F3D-9928-A740FFBC96C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81651B8D-AAEF-41DB-B434-76DFE2CA98B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -485,8 +485,11 @@
   <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>